<commit_message>
Update schedule file: Y5_B2526_General_&_Special_Internal_2_B1_schedule.xlsx
</commit_message>
<xml_diff>
--- a/modules_schedules/Y5_B2526_General_&_Special_Internal_2_B1_schedule.xlsx
+++ b/modules_schedules/Y5_B2526_General_&_Special_Internal_2_B1_schedule.xlsx
@@ -520,12 +520,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -555,12 +555,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -625,12 +625,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -835,12 +835,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>gastroenterology</t>
+          <t>endocrinology</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>nephrology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>nephrology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -940,12 +940,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>nephrology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -975,12 +975,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>nephrology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1010,12 +1010,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>nephrology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1080,22 +1080,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1115,22 +1115,22 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1185,22 +1185,22 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>gastroenterology</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1220,22 +1220,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>nephrology</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1255,22 +1255,22 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>nephrology</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1290,22 +1290,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>nephrology</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1325,22 +1325,22 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>physical medicine</t>
+          <t>nephrology</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -1360,22 +1360,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>physical medicine</t>
+          <t>nephrology</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1395,12 +1395,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>rheumatology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>rheumatology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>rheumatology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>rheumatology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1535,12 +1535,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1A1</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>rheumatology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -1575,17 +1575,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1610,17 +1610,17 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>neurology</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1680,17 +1680,17 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>physical medicine</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -1715,17 +1715,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>physical medicine</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1750,17 +1750,17 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>rheumatology</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -1785,17 +1785,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>rheumatology</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1820,17 +1820,17 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>rheumatology</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -1855,17 +1855,17 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>rheumatology</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -1890,17 +1890,17 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>endocrinology</t>
+          <t>rheumatology</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">

</xml_diff>